<commit_message>
feat: Remove PDF to image conversion functionality and associated metadata.
</commit_message>
<xml_diff>
--- a/data/out/mitsumori/mitsumori.xlsx
+++ b/data/out/mitsumori/mitsumori.xlsx
@@ -9,7 +9,6 @@
   <sheets>
     <sheet name="変換結果" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="フォント・カラー情報" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="PDF画像" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="17">
+  <fonts count="16">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -99,10 +98,6 @@
     <font>
       <b val="1"/>
       <sz val="11"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <sz val="12"/>
     </font>
   </fonts>
   <fills count="5">
@@ -242,7 +237,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -323,7 +318,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -398,36 +392,6 @@
     </indexedColors>
   </colors>
 </styleSheet>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <oneCellAnchor>
-    <from>
-      <col>0</col>
-      <colOff>0</colOff>
-      <row>1</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="5715000" cy="8086725"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="1" name="Image 1" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId1"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -5623,26 +5587,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:A1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="38" t="inlineStr">
-        <is>
-          <t>Page 1</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
feat: Enhance data extraction to include page dimensions and standardize font names across outputs.
</commit_message>
<xml_diff>
--- a/data/out/mitsumori/mitsumori.xlsx
+++ b/data/out/mitsumori/mitsumori.xlsx
@@ -10,7 +10,9 @@
     <sheet name="変換結果" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="フォント・カラー情報" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'変換結果'!$A$1:$DP$182</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -18,13 +20,17 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="16">
+  <fonts count="17">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="11"/>
     </font>
     <font>
       <name val="MS-Mincho"/>
@@ -235,13 +241,13 @@
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -251,70 +257,70 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -686,138 +692,138 @@
   <dimension ref="F10:DI165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="0.9399999999999999" customWidth="1" min="1" max="1"/>
-    <col width="0.9399999999999999" customWidth="1" min="2" max="2"/>
-    <col width="0.9399999999999999" customWidth="1" min="3" max="3"/>
-    <col width="0.9399999999999999" customWidth="1" min="4" max="4"/>
-    <col width="0.9399999999999999" customWidth="1" min="5" max="5"/>
-    <col width="0.9399999999999999" customWidth="1" min="6" max="6"/>
-    <col width="0.9399999999999999" customWidth="1" min="7" max="7"/>
-    <col width="0.9399999999999999" customWidth="1" min="8" max="8"/>
-    <col width="0.9399999999999999" customWidth="1" min="9" max="9"/>
-    <col width="0.9399999999999999" customWidth="1" min="10" max="10"/>
-    <col width="0.9399999999999999" customWidth="1" min="11" max="11"/>
-    <col width="0.9399999999999999" customWidth="1" min="12" max="12"/>
-    <col width="0.9399999999999999" customWidth="1" min="13" max="13"/>
-    <col width="0.9399999999999999" customWidth="1" min="14" max="14"/>
-    <col width="0.9399999999999999" customWidth="1" min="15" max="15"/>
-    <col width="0.9399999999999999" customWidth="1" min="16" max="16"/>
-    <col width="0.9399999999999999" customWidth="1" min="17" max="17"/>
-    <col width="0.9399999999999999" customWidth="1" min="18" max="18"/>
-    <col width="0.9399999999999999" customWidth="1" min="19" max="19"/>
-    <col width="0.9399999999999999" customWidth="1" min="20" max="20"/>
-    <col width="0.9399999999999999" customWidth="1" min="21" max="21"/>
-    <col width="0.9399999999999999" customWidth="1" min="22" max="22"/>
-    <col width="0.9399999999999999" customWidth="1" min="23" max="23"/>
-    <col width="0.9399999999999999" customWidth="1" min="24" max="24"/>
-    <col width="0.9399999999999999" customWidth="1" min="25" max="25"/>
-    <col width="0.9399999999999999" customWidth="1" min="26" max="26"/>
-    <col width="0.9399999999999999" customWidth="1" min="27" max="27"/>
-    <col width="0.9399999999999999" customWidth="1" min="28" max="28"/>
-    <col width="0.9399999999999999" customWidth="1" min="29" max="29"/>
-    <col width="0.9399999999999999" customWidth="1" min="30" max="30"/>
-    <col width="0.9399999999999999" customWidth="1" min="31" max="31"/>
-    <col width="0.9399999999999999" customWidth="1" min="32" max="32"/>
-    <col width="0.9399999999999999" customWidth="1" min="33" max="33"/>
-    <col width="0.9399999999999999" customWidth="1" min="34" max="34"/>
-    <col width="0.9399999999999999" customWidth="1" min="35" max="35"/>
-    <col width="0.9399999999999999" customWidth="1" min="36" max="36"/>
-    <col width="0.9399999999999999" customWidth="1" min="37" max="37"/>
-    <col width="0.9399999999999999" customWidth="1" min="38" max="38"/>
-    <col width="0.9399999999999999" customWidth="1" min="39" max="39"/>
-    <col width="0.9399999999999999" customWidth="1" min="40" max="40"/>
-    <col width="0.9399999999999999" customWidth="1" min="41" max="41"/>
-    <col width="0.9399999999999999" customWidth="1" min="42" max="42"/>
-    <col width="0.9399999999999999" customWidth="1" min="43" max="43"/>
-    <col width="0.9399999999999999" customWidth="1" min="44" max="44"/>
-    <col width="0.9399999999999999" customWidth="1" min="45" max="45"/>
-    <col width="0.9399999999999999" customWidth="1" min="46" max="46"/>
-    <col width="0.9399999999999999" customWidth="1" min="47" max="47"/>
-    <col width="0.9399999999999999" customWidth="1" min="48" max="48"/>
-    <col width="0.9399999999999999" customWidth="1" min="49" max="49"/>
-    <col width="0.9399999999999999" customWidth="1" min="50" max="50"/>
-    <col width="0.9399999999999999" customWidth="1" min="51" max="51"/>
-    <col width="0.9399999999999999" customWidth="1" min="52" max="52"/>
-    <col width="0.9399999999999999" customWidth="1" min="53" max="53"/>
-    <col width="0.9399999999999999" customWidth="1" min="54" max="54"/>
-    <col width="0.9399999999999999" customWidth="1" min="55" max="55"/>
-    <col width="0.9399999999999999" customWidth="1" min="56" max="56"/>
-    <col width="0.9399999999999999" customWidth="1" min="57" max="57"/>
-    <col width="0.9399999999999999" customWidth="1" min="58" max="58"/>
-    <col width="0.9399999999999999" customWidth="1" min="59" max="59"/>
-    <col width="0.9399999999999999" customWidth="1" min="60" max="60"/>
-    <col width="0.9399999999999999" customWidth="1" min="61" max="61"/>
-    <col width="0.9399999999999999" customWidth="1" min="62" max="62"/>
-    <col width="0.9399999999999999" customWidth="1" min="63" max="63"/>
-    <col width="0.9399999999999999" customWidth="1" min="64" max="64"/>
-    <col width="0.9399999999999999" customWidth="1" min="65" max="65"/>
-    <col width="0.9399999999999999" customWidth="1" min="66" max="66"/>
-    <col width="0.9399999999999999" customWidth="1" min="67" max="67"/>
-    <col width="0.9399999999999999" customWidth="1" min="68" max="68"/>
-    <col width="0.9399999999999999" customWidth="1" min="69" max="69"/>
-    <col width="0.9399999999999999" customWidth="1" min="70" max="70"/>
-    <col width="0.9399999999999999" customWidth="1" min="71" max="71"/>
-    <col width="0.9399999999999999" customWidth="1" min="72" max="72"/>
-    <col width="0.9399999999999999" customWidth="1" min="73" max="73"/>
-    <col width="0.9399999999999999" customWidth="1" min="74" max="74"/>
-    <col width="0.9399999999999999" customWidth="1" min="75" max="75"/>
-    <col width="0.9399999999999999" customWidth="1" min="76" max="76"/>
-    <col width="0.9399999999999999" customWidth="1" min="77" max="77"/>
-    <col width="0.9399999999999999" customWidth="1" min="78" max="78"/>
-    <col width="0.9399999999999999" customWidth="1" min="79" max="79"/>
-    <col width="0.9399999999999999" customWidth="1" min="80" max="80"/>
-    <col width="0.9399999999999999" customWidth="1" min="81" max="81"/>
-    <col width="0.9399999999999999" customWidth="1" min="82" max="82"/>
-    <col width="0.9399999999999999" customWidth="1" min="83" max="83"/>
-    <col width="0.9399999999999999" customWidth="1" min="84" max="84"/>
-    <col width="0.9399999999999999" customWidth="1" min="85" max="85"/>
-    <col width="0.9399999999999999" customWidth="1" min="86" max="86"/>
-    <col width="0.9399999999999999" customWidth="1" min="87" max="87"/>
-    <col width="0.9399999999999999" customWidth="1" min="88" max="88"/>
-    <col width="0.9399999999999999" customWidth="1" min="89" max="89"/>
-    <col width="0.9399999999999999" customWidth="1" min="90" max="90"/>
-    <col width="0.9399999999999999" customWidth="1" min="91" max="91"/>
-    <col width="0.9399999999999999" customWidth="1" min="92" max="92"/>
-    <col width="0.9399999999999999" customWidth="1" min="93" max="93"/>
-    <col width="0.9399999999999999" customWidth="1" min="94" max="94"/>
-    <col width="0.9399999999999999" customWidth="1" min="95" max="95"/>
-    <col width="0.9399999999999999" customWidth="1" min="96" max="96"/>
-    <col width="0.9399999999999999" customWidth="1" min="97" max="97"/>
-    <col width="0.9399999999999999" customWidth="1" min="98" max="98"/>
-    <col width="0.9399999999999999" customWidth="1" min="99" max="99"/>
-    <col width="0.9399999999999999" customWidth="1" min="100" max="100"/>
-    <col width="0.9399999999999999" customWidth="1" min="101" max="101"/>
-    <col width="0.9399999999999999" customWidth="1" min="102" max="102"/>
-    <col width="0.9399999999999999" customWidth="1" min="103" max="103"/>
-    <col width="0.9399999999999999" customWidth="1" min="104" max="104"/>
-    <col width="0.9399999999999999" customWidth="1" min="105" max="105"/>
-    <col width="0.9399999999999999" customWidth="1" min="106" max="106"/>
-    <col width="0.9399999999999999" customWidth="1" min="107" max="107"/>
-    <col width="0.9399999999999999" customWidth="1" min="108" max="108"/>
-    <col width="0.9399999999999999" customWidth="1" min="109" max="109"/>
-    <col width="0.9399999999999999" customWidth="1" min="110" max="110"/>
-    <col width="0.9399999999999999" customWidth="1" min="111" max="111"/>
-    <col width="0.9399999999999999" customWidth="1" min="112" max="112"/>
-    <col width="0.9399999999999999" customWidth="1" min="113" max="113"/>
-    <col width="0.9399999999999999" customWidth="1" min="114" max="114"/>
-    <col width="0.9399999999999999" customWidth="1" min="115" max="115"/>
-    <col width="0.9399999999999999" customWidth="1" min="116" max="116"/>
-    <col width="0.9399999999999999" customWidth="1" min="117" max="117"/>
-    <col width="0.9399999999999999" customWidth="1" min="118" max="118"/>
-    <col width="0.9399999999999999" customWidth="1" min="119" max="119"/>
-    <col width="0.9399999999999999" customWidth="1" min="120" max="120"/>
+    <col width="0.75" customWidth="1" min="1" max="1"/>
+    <col width="0.75" customWidth="1" min="2" max="2"/>
+    <col width="0.75" customWidth="1" min="3" max="3"/>
+    <col width="0.75" customWidth="1" min="4" max="4"/>
+    <col width="0.75" customWidth="1" min="5" max="5"/>
+    <col width="0.75" customWidth="1" min="6" max="6"/>
+    <col width="0.75" customWidth="1" min="7" max="7"/>
+    <col width="0.75" customWidth="1" min="8" max="8"/>
+    <col width="0.75" customWidth="1" min="9" max="9"/>
+    <col width="0.75" customWidth="1" min="10" max="10"/>
+    <col width="0.75" customWidth="1" min="11" max="11"/>
+    <col width="0.75" customWidth="1" min="12" max="12"/>
+    <col width="0.75" customWidth="1" min="13" max="13"/>
+    <col width="0.75" customWidth="1" min="14" max="14"/>
+    <col width="0.75" customWidth="1" min="15" max="15"/>
+    <col width="0.75" customWidth="1" min="16" max="16"/>
+    <col width="0.75" customWidth="1" min="17" max="17"/>
+    <col width="0.75" customWidth="1" min="18" max="18"/>
+    <col width="0.75" customWidth="1" min="19" max="19"/>
+    <col width="0.75" customWidth="1" min="20" max="20"/>
+    <col width="0.75" customWidth="1" min="21" max="21"/>
+    <col width="0.75" customWidth="1" min="22" max="22"/>
+    <col width="0.75" customWidth="1" min="23" max="23"/>
+    <col width="0.75" customWidth="1" min="24" max="24"/>
+    <col width="0.75" customWidth="1" min="25" max="25"/>
+    <col width="0.75" customWidth="1" min="26" max="26"/>
+    <col width="0.75" customWidth="1" min="27" max="27"/>
+    <col width="0.75" customWidth="1" min="28" max="28"/>
+    <col width="0.75" customWidth="1" min="29" max="29"/>
+    <col width="0.75" customWidth="1" min="30" max="30"/>
+    <col width="0.75" customWidth="1" min="31" max="31"/>
+    <col width="0.75" customWidth="1" min="32" max="32"/>
+    <col width="0.75" customWidth="1" min="33" max="33"/>
+    <col width="0.75" customWidth="1" min="34" max="34"/>
+    <col width="0.75" customWidth="1" min="35" max="35"/>
+    <col width="0.75" customWidth="1" min="36" max="36"/>
+    <col width="0.75" customWidth="1" min="37" max="37"/>
+    <col width="0.75" customWidth="1" min="38" max="38"/>
+    <col width="0.75" customWidth="1" min="39" max="39"/>
+    <col width="0.75" customWidth="1" min="40" max="40"/>
+    <col width="0.75" customWidth="1" min="41" max="41"/>
+    <col width="0.75" customWidth="1" min="42" max="42"/>
+    <col width="0.75" customWidth="1" min="43" max="43"/>
+    <col width="0.75" customWidth="1" min="44" max="44"/>
+    <col width="0.75" customWidth="1" min="45" max="45"/>
+    <col width="0.75" customWidth="1" min="46" max="46"/>
+    <col width="0.75" customWidth="1" min="47" max="47"/>
+    <col width="0.75" customWidth="1" min="48" max="48"/>
+    <col width="0.75" customWidth="1" min="49" max="49"/>
+    <col width="0.75" customWidth="1" min="50" max="50"/>
+    <col width="0.75" customWidth="1" min="51" max="51"/>
+    <col width="0.75" customWidth="1" min="52" max="52"/>
+    <col width="0.75" customWidth="1" min="53" max="53"/>
+    <col width="0.75" customWidth="1" min="54" max="54"/>
+    <col width="0.75" customWidth="1" min="55" max="55"/>
+    <col width="0.75" customWidth="1" min="56" max="56"/>
+    <col width="0.75" customWidth="1" min="57" max="57"/>
+    <col width="0.75" customWidth="1" min="58" max="58"/>
+    <col width="0.75" customWidth="1" min="59" max="59"/>
+    <col width="0.75" customWidth="1" min="60" max="60"/>
+    <col width="0.75" customWidth="1" min="61" max="61"/>
+    <col width="0.75" customWidth="1" min="62" max="62"/>
+    <col width="0.75" customWidth="1" min="63" max="63"/>
+    <col width="0.75" customWidth="1" min="64" max="64"/>
+    <col width="0.75" customWidth="1" min="65" max="65"/>
+    <col width="0.75" customWidth="1" min="66" max="66"/>
+    <col width="0.75" customWidth="1" min="67" max="67"/>
+    <col width="0.75" customWidth="1" min="68" max="68"/>
+    <col width="0.75" customWidth="1" min="69" max="69"/>
+    <col width="0.75" customWidth="1" min="70" max="70"/>
+    <col width="0.75" customWidth="1" min="71" max="71"/>
+    <col width="0.75" customWidth="1" min="72" max="72"/>
+    <col width="0.75" customWidth="1" min="73" max="73"/>
+    <col width="0.75" customWidth="1" min="74" max="74"/>
+    <col width="0.75" customWidth="1" min="75" max="75"/>
+    <col width="0.75" customWidth="1" min="76" max="76"/>
+    <col width="0.75" customWidth="1" min="77" max="77"/>
+    <col width="0.75" customWidth="1" min="78" max="78"/>
+    <col width="0.75" customWidth="1" min="79" max="79"/>
+    <col width="0.75" customWidth="1" min="80" max="80"/>
+    <col width="0.75" customWidth="1" min="81" max="81"/>
+    <col width="0.75" customWidth="1" min="82" max="82"/>
+    <col width="0.75" customWidth="1" min="83" max="83"/>
+    <col width="0.75" customWidth="1" min="84" max="84"/>
+    <col width="0.75" customWidth="1" min="85" max="85"/>
+    <col width="0.75" customWidth="1" min="86" max="86"/>
+    <col width="0.75" customWidth="1" min="87" max="87"/>
+    <col width="0.75" customWidth="1" min="88" max="88"/>
+    <col width="0.75" customWidth="1" min="89" max="89"/>
+    <col width="0.75" customWidth="1" min="90" max="90"/>
+    <col width="0.75" customWidth="1" min="91" max="91"/>
+    <col width="0.75" customWidth="1" min="92" max="92"/>
+    <col width="0.75" customWidth="1" min="93" max="93"/>
+    <col width="0.75" customWidth="1" min="94" max="94"/>
+    <col width="0.75" customWidth="1" min="95" max="95"/>
+    <col width="0.75" customWidth="1" min="96" max="96"/>
+    <col width="0.75" customWidth="1" min="97" max="97"/>
+    <col width="0.75" customWidth="1" min="98" max="98"/>
+    <col width="0.75" customWidth="1" min="99" max="99"/>
+    <col width="0.75" customWidth="1" min="100" max="100"/>
+    <col width="0.75" customWidth="1" min="101" max="101"/>
+    <col width="0.75" customWidth="1" min="102" max="102"/>
+    <col width="0.75" customWidth="1" min="103" max="103"/>
+    <col width="0.75" customWidth="1" min="104" max="104"/>
+    <col width="0.75" customWidth="1" min="105" max="105"/>
+    <col width="0.75" customWidth="1" min="106" max="106"/>
+    <col width="0.75" customWidth="1" min="107" max="107"/>
+    <col width="0.75" customWidth="1" min="108" max="108"/>
+    <col width="0.75" customWidth="1" min="109" max="109"/>
+    <col width="0.75" customWidth="1" min="110" max="110"/>
+    <col width="0.75" customWidth="1" min="111" max="111"/>
+    <col width="0.75" customWidth="1" min="112" max="112"/>
+    <col width="0.75" customWidth="1" min="113" max="113"/>
+    <col width="0.75" customWidth="1" min="114" max="114"/>
+    <col width="0.75" customWidth="1" min="115" max="115"/>
+    <col width="0.75" customWidth="1" min="116" max="116"/>
+    <col width="0.75" customWidth="1" min="117" max="117"/>
+    <col width="0.75" customWidth="1" min="118" max="118"/>
+    <col width="0.75" customWidth="1" min="119" max="119"/>
+    <col width="0.75" customWidth="1" min="120" max="120"/>
   </cols>
   <sheetData>
-    <row r="1" ht="4.96" customHeight="1"/>
-    <row r="2" ht="4.96" customHeight="1"/>
-    <row r="3" ht="4.96" customHeight="1"/>
-    <row r="4" ht="4.96" customHeight="1"/>
-    <row r="5" ht="4.96" customHeight="1"/>
-    <row r="6" ht="4.96" customHeight="1"/>
-    <row r="7" ht="4.96" customHeight="1"/>
-    <row r="8" ht="4.96" customHeight="1"/>
-    <row r="9" ht="4.96" customHeight="1"/>
-    <row r="10" ht="4.96" customHeight="1">
+    <row r="1" ht="4.65" customHeight="1"/>
+    <row r="2" ht="4.65" customHeight="1"/>
+    <row r="3" ht="4.65" customHeight="1"/>
+    <row r="4" ht="4.65" customHeight="1"/>
+    <row r="5" ht="4.65" customHeight="1"/>
+    <row r="6" ht="4.65" customHeight="1"/>
+    <row r="7" ht="4.65" customHeight="1"/>
+    <row r="8" ht="4.65" customHeight="1"/>
+    <row r="9" ht="4.65" customHeight="1"/>
+    <row r="10" ht="4.65" customHeight="1">
       <c r="AT10" s="1" t="n"/>
       <c r="AU10" s="2" t="n"/>
       <c r="AV10" s="2" t="n"/>
@@ -855,7 +861,7 @@
       <c r="BX10" s="2" t="n"/>
       <c r="BY10" s="4" t="n"/>
     </row>
-    <row r="11" ht="4.96" customHeight="1">
+    <row r="11" ht="4.65" customHeight="1">
       <c r="AT11" s="5" t="n"/>
       <c r="AU11" s="6" t="n"/>
       <c r="AV11" s="6" t="n"/>
@@ -889,7 +895,7 @@
       <c r="BX11" s="6" t="n"/>
       <c r="BY11" s="7" t="n"/>
     </row>
-    <row r="12" ht="4.96" customHeight="1">
+    <row r="12" ht="4.65" customHeight="1">
       <c r="AT12" s="5" t="n"/>
       <c r="AU12" s="6" t="n"/>
       <c r="AV12" s="6" t="n"/>
@@ -923,7 +929,7 @@
       <c r="BX12" s="6" t="n"/>
       <c r="BY12" s="7" t="n"/>
     </row>
-    <row r="13" ht="4.96" customHeight="1">
+    <row r="13" ht="4.65" customHeight="1">
       <c r="AT13" s="5" t="n"/>
       <c r="AU13" s="6" t="n"/>
       <c r="AV13" s="6" t="n"/>
@@ -957,7 +963,7 @@
       <c r="BX13" s="6" t="n"/>
       <c r="BY13" s="7" t="n"/>
     </row>
-    <row r="14" ht="4.96" customHeight="1">
+    <row r="14" ht="4.65" customHeight="1">
       <c r="AT14" s="5" t="n"/>
       <c r="AU14" s="6" t="n"/>
       <c r="AV14" s="6" t="n"/>
@@ -991,7 +997,7 @@
       <c r="BX14" s="6" t="n"/>
       <c r="BY14" s="7" t="n"/>
     </row>
-    <row r="15" ht="4.96" customHeight="1">
+    <row r="15" ht="4.65" customHeight="1">
       <c r="AT15" s="5" t="n"/>
       <c r="AU15" s="6" t="n"/>
       <c r="AV15" s="6" t="n"/>
@@ -1025,7 +1031,7 @@
       <c r="BX15" s="6" t="n"/>
       <c r="BY15" s="7" t="n"/>
     </row>
-    <row r="16" ht="4.96" customHeight="1">
+    <row r="16" ht="4.65" customHeight="1">
       <c r="AT16" s="8" t="n"/>
       <c r="AU16" s="9" t="n"/>
       <c r="AV16" s="9" t="n"/>
@@ -1059,10 +1065,10 @@
       <c r="BX16" s="9" t="n"/>
       <c r="BY16" s="10" t="n"/>
     </row>
-    <row r="17" ht="4.96" customHeight="1"/>
-    <row r="18" ht="4.96" customHeight="1"/>
-    <row r="19" ht="4.96" customHeight="1"/>
-    <row r="20" ht="4.96" customHeight="1">
+    <row r="17" ht="4.65" customHeight="1"/>
+    <row r="18" ht="4.65" customHeight="1"/>
+    <row r="19" ht="4.65" customHeight="1"/>
+    <row r="20" ht="4.65" customHeight="1">
       <c r="CC20" s="11" t="inlineStr">
         <is>
           <t>見積書Ｎｏ．</t>
@@ -1074,8 +1080,8 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="4.96" customHeight="1"/>
-    <row r="22" ht="4.96" customHeight="1">
+    <row r="21" ht="4.65" customHeight="1"/>
+    <row r="22" ht="4.65" customHeight="1">
       <c r="G22" s="12" t="inlineStr">
         <is>
           <t>△△株式会社</t>
@@ -1117,9 +1123,9 @@
       <c r="DD22" s="2" t="n"/>
       <c r="DE22" s="2" t="n"/>
     </row>
-    <row r="23" ht="4.96" customHeight="1"/>
-    <row r="24" ht="4.96" customHeight="1"/>
-    <row r="25" ht="4.96" customHeight="1">
+    <row r="23" ht="4.65" customHeight="1"/>
+    <row r="24" ht="4.65" customHeight="1"/>
+    <row r="25" ht="4.65" customHeight="1">
       <c r="F25" s="2" t="n"/>
       <c r="G25" s="2" t="n"/>
       <c r="H25" s="2" t="n"/>
@@ -1178,7 +1184,7 @@
       <c r="BI25" s="2" t="n"/>
       <c r="BJ25" s="2" t="n"/>
     </row>
-    <row r="26" ht="4.96" customHeight="1">
+    <row r="26" ht="4.65" customHeight="1">
       <c r="CC26" s="11" t="inlineStr">
         <is>
           <t>作成日:</t>
@@ -1190,9 +1196,9 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="4.96" customHeight="1"/>
-    <row r="28" ht="4.96" customHeight="1"/>
-    <row r="29" ht="4.96" customHeight="1">
+    <row r="27" ht="4.65" customHeight="1"/>
+    <row r="28" ht="4.65" customHeight="1"/>
+    <row r="29" ht="4.65" customHeight="1">
       <c r="CB29" s="2" t="n"/>
       <c r="CC29" s="2" t="n"/>
       <c r="CD29" s="2" t="n"/>
@@ -1223,30 +1229,30 @@
       <c r="DC29" s="2" t="n"/>
       <c r="DD29" s="2" t="n"/>
     </row>
-    <row r="30" ht="4.96" customHeight="1"/>
-    <row r="31" ht="4.96" customHeight="1">
+    <row r="30" ht="4.65" customHeight="1"/>
+    <row r="31" ht="4.65" customHeight="1">
       <c r="O31" s="13" t="inlineStr">
         <is>
           <t>下記のとおり御見積申し上げます。</t>
         </is>
       </c>
     </row>
-    <row r="32" ht="4.96" customHeight="1"/>
-    <row r="33" ht="4.96" customHeight="1"/>
-    <row r="34" ht="4.96" customHeight="1">
+    <row r="32" ht="4.65" customHeight="1"/>
+    <row r="33" ht="4.65" customHeight="1"/>
+    <row r="34" ht="4.65" customHeight="1">
       <c r="O34" s="13" t="inlineStr">
         <is>
           <t>何卒ご用命の程、お願い申し上げます。</t>
         </is>
       </c>
     </row>
-    <row r="35" ht="4.96" customHeight="1"/>
-    <row r="36" ht="4.96" customHeight="1"/>
-    <row r="37" ht="4.96" customHeight="1"/>
-    <row r="38" ht="4.96" customHeight="1"/>
-    <row r="39" ht="4.96" customHeight="1"/>
-    <row r="40" ht="4.96" customHeight="1"/>
-    <row r="41" ht="4.96" customHeight="1">
+    <row r="35" ht="4.65" customHeight="1"/>
+    <row r="36" ht="4.65" customHeight="1"/>
+    <row r="37" ht="4.65" customHeight="1"/>
+    <row r="38" ht="4.65" customHeight="1"/>
+    <row r="39" ht="4.65" customHeight="1"/>
+    <row r="40" ht="4.65" customHeight="1"/>
+    <row r="41" ht="4.65" customHeight="1">
       <c r="F41" s="13" t="inlineStr">
         <is>
           <t>受渡期日:</t>
@@ -1258,15 +1264,15 @@
         </is>
       </c>
     </row>
-    <row r="42" ht="4.96" customHeight="1">
+    <row r="42" ht="4.65" customHeight="1">
       <c r="CC42" s="14" t="inlineStr">
         <is>
           <t xml:space="preserve">ワークフロー商事株式会社 </t>
         </is>
       </c>
     </row>
-    <row r="43" ht="4.96" customHeight="1"/>
-    <row r="44" ht="4.96" customHeight="1">
+    <row r="43" ht="4.65" customHeight="1"/>
+    <row r="44" ht="4.65" customHeight="1">
       <c r="F44" s="2" t="n"/>
       <c r="G44" s="2" t="n"/>
       <c r="H44" s="2" t="n"/>
@@ -1325,8 +1331,8 @@
       <c r="BI44" s="2" t="n"/>
       <c r="BJ44" s="2" t="n"/>
     </row>
-    <row r="45" ht="4.96" customHeight="1"/>
-    <row r="46" ht="4.96" customHeight="1">
+    <row r="45" ht="4.65" customHeight="1"/>
+    <row r="46" ht="4.65" customHeight="1">
       <c r="F46" s="13" t="inlineStr">
         <is>
           <t>取引方法:</t>
@@ -1343,9 +1349,9 @@
         </is>
       </c>
     </row>
-    <row r="47" ht="4.96" customHeight="1"/>
-    <row r="48" ht="4.96" customHeight="1"/>
-    <row r="49" ht="4.96" customHeight="1">
+    <row r="47" ht="4.65" customHeight="1"/>
+    <row r="48" ht="4.65" customHeight="1"/>
+    <row r="49" ht="4.65" customHeight="1">
       <c r="F49" s="2" t="n"/>
       <c r="G49" s="2" t="n"/>
       <c r="H49" s="2" t="n"/>
@@ -1409,8 +1415,8 @@
         </is>
       </c>
     </row>
-    <row r="50" ht="4.96" customHeight="1"/>
-    <row r="51" ht="4.96" customHeight="1">
+    <row r="50" ht="4.65" customHeight="1"/>
+    <row r="51" ht="4.65" customHeight="1">
       <c r="F51" s="13" t="inlineStr">
         <is>
           <t>有効期限:</t>
@@ -1427,9 +1433,9 @@
         </is>
       </c>
     </row>
-    <row r="52" ht="4.96" customHeight="1"/>
-    <row r="53" ht="4.96" customHeight="1"/>
-    <row r="54" ht="4.96" customHeight="1">
+    <row r="52" ht="4.65" customHeight="1"/>
+    <row r="53" ht="4.65" customHeight="1"/>
+    <row r="54" ht="4.65" customHeight="1">
       <c r="F54" s="2" t="n"/>
       <c r="G54" s="2" t="n"/>
       <c r="H54" s="2" t="n"/>
@@ -1493,22 +1499,22 @@
         </is>
       </c>
     </row>
-    <row r="55" ht="4.96" customHeight="1"/>
-    <row r="56" ht="4.96" customHeight="1">
+    <row r="55" ht="4.65" customHeight="1"/>
+    <row r="56" ht="4.65" customHeight="1">
       <c r="CD56" s="11" t="inlineStr">
         <is>
           <t> </t>
         </is>
       </c>
     </row>
-    <row r="57" ht="4.96" customHeight="1">
+    <row r="57" ht="4.65" customHeight="1">
       <c r="F57" s="13" t="inlineStr">
         <is>
           <t>貴社管理番号：</t>
         </is>
       </c>
     </row>
-    <row r="58" ht="4.96" customHeight="1">
+    <row r="58" ht="4.65" customHeight="1">
       <c r="CM58" s="1" t="n"/>
       <c r="CN58" s="2" t="n"/>
       <c r="CO58" s="2" t="n"/>
@@ -1531,7 +1537,7 @@
       <c r="DF58" s="2" t="n"/>
       <c r="DG58" s="1" t="n"/>
     </row>
-    <row r="59" ht="4.96" customHeight="1">
+    <row r="59" ht="4.65" customHeight="1">
       <c r="CM59" s="5" t="n"/>
       <c r="CP59" s="15" t="inlineStr">
         <is>
@@ -1546,7 +1552,7 @@
       </c>
       <c r="DG59" s="5" t="n"/>
     </row>
-    <row r="60" ht="4.96" customHeight="1">
+    <row r="60" ht="4.65" customHeight="1">
       <c r="F60" s="2" t="n"/>
       <c r="G60" s="2" t="n"/>
       <c r="H60" s="2" t="n"/>
@@ -1612,42 +1618,42 @@
       <c r="DF60" s="2" t="n"/>
       <c r="DG60" s="1" t="n"/>
     </row>
-    <row r="61" ht="4.96" customHeight="1">
+    <row r="61" ht="4.65" customHeight="1">
       <c r="CM61" s="5" t="n"/>
       <c r="CW61" s="5" t="n"/>
       <c r="DG61" s="5" t="n"/>
     </row>
-    <row r="62" ht="4.96" customHeight="1">
+    <row r="62" ht="4.65" customHeight="1">
       <c r="CM62" s="5" t="n"/>
       <c r="CW62" s="5" t="n"/>
       <c r="DG62" s="5" t="n"/>
     </row>
-    <row r="63" ht="4.96" customHeight="1">
+    <row r="63" ht="4.65" customHeight="1">
       <c r="CM63" s="5" t="n"/>
       <c r="CW63" s="5" t="n"/>
       <c r="DG63" s="5" t="n"/>
     </row>
-    <row r="64" ht="4.96" customHeight="1">
+    <row r="64" ht="4.65" customHeight="1">
       <c r="CM64" s="5" t="n"/>
       <c r="CW64" s="5" t="n"/>
       <c r="DG64" s="5" t="n"/>
     </row>
-    <row r="65" ht="4.96" customHeight="1">
+    <row r="65" ht="4.65" customHeight="1">
       <c r="CM65" s="5" t="n"/>
       <c r="CW65" s="5" t="n"/>
       <c r="DG65" s="5" t="n"/>
     </row>
-    <row r="66" ht="4.96" customHeight="1">
+    <row r="66" ht="4.65" customHeight="1">
       <c r="CM66" s="5" t="n"/>
       <c r="CW66" s="5" t="n"/>
       <c r="DG66" s="5" t="n"/>
     </row>
-    <row r="67" ht="4.96" customHeight="1">
+    <row r="67" ht="4.65" customHeight="1">
       <c r="CM67" s="5" t="n"/>
       <c r="CW67" s="5" t="n"/>
       <c r="DG67" s="5" t="n"/>
     </row>
-    <row r="68" ht="4.96" customHeight="1">
+    <row r="68" ht="4.65" customHeight="1">
       <c r="CM68" s="1" t="n"/>
       <c r="CN68" s="2" t="n"/>
       <c r="CO68" s="2" t="n"/>
@@ -1670,14 +1676,14 @@
       <c r="DF68" s="2" t="n"/>
       <c r="DG68" s="1" t="n"/>
     </row>
-    <row r="69" ht="4.96" customHeight="1">
+    <row r="69" ht="4.65" customHeight="1">
       <c r="AY69" s="16" t="inlineStr">
         <is>
           <t>\3,700,000</t>
         </is>
       </c>
     </row>
-    <row r="70" ht="4.96" customHeight="1">
+    <row r="70" ht="4.65" customHeight="1">
       <c r="W70" s="17" t="inlineStr">
         <is>
           <t>合計金額：</t>
@@ -1689,10 +1695,10 @@
         </is>
       </c>
     </row>
-    <row r="71" ht="4.96" customHeight="1"/>
-    <row r="72" ht="4.96" customHeight="1"/>
-    <row r="73" ht="4.96" customHeight="1"/>
-    <row r="74" ht="4.96" customHeight="1">
+    <row r="71" ht="4.65" customHeight="1"/>
+    <row r="72" ht="4.65" customHeight="1"/>
+    <row r="73" ht="4.65" customHeight="1"/>
+    <row r="74" ht="4.65" customHeight="1">
       <c r="L74" s="19" t="n"/>
       <c r="M74" s="19" t="n"/>
       <c r="N74" s="19" t="n"/>
@@ -1796,9 +1802,9 @@
       <c r="DH74" s="19" t="n"/>
       <c r="DI74" s="19" t="n"/>
     </row>
-    <row r="75" ht="4.96" customHeight="1"/>
-    <row r="76" ht="4.96" customHeight="1"/>
-    <row r="77" ht="4.96" customHeight="1">
+    <row r="75" ht="4.65" customHeight="1"/>
+    <row r="76" ht="4.65" customHeight="1"/>
+    <row r="77" ht="4.65" customHeight="1">
       <c r="L77" s="20" t="inlineStr">
         <is>
           <t>No.</t>
@@ -1926,7 +1932,7 @@
       <c r="DH77" s="2" t="n"/>
       <c r="DI77" s="1" t="n"/>
     </row>
-    <row r="78" ht="4.96" customHeight="1">
+    <row r="78" ht="4.65" customHeight="1">
       <c r="L78" s="5" t="n"/>
       <c r="P78" s="5" t="n"/>
       <c r="BK78" s="5" t="n"/>
@@ -1935,7 +1941,7 @@
       <c r="CT78" s="5" t="n"/>
       <c r="DI78" s="5" t="n"/>
     </row>
-    <row r="79" ht="4.96" customHeight="1">
+    <row r="79" ht="4.65" customHeight="1">
       <c r="L79" s="1" t="n"/>
       <c r="M79" s="2" t="n"/>
       <c r="N79" s="2" t="n"/>
@@ -2039,7 +2045,7 @@
       <c r="DH79" s="2" t="n"/>
       <c r="DI79" s="1" t="n"/>
     </row>
-    <row r="80" ht="4.96" customHeight="1">
+    <row r="80" ht="4.65" customHeight="1">
       <c r="L80" s="1" t="n"/>
       <c r="M80" s="2" t="n"/>
       <c r="N80" s="2" t="n"/>
@@ -2143,7 +2149,7 @@
       <c r="DH80" s="2" t="n"/>
       <c r="DI80" s="1" t="n"/>
     </row>
-    <row r="81" ht="4.96" customHeight="1">
+    <row r="81" ht="4.65" customHeight="1">
       <c r="L81" s="5" t="n"/>
       <c r="M81" s="22" t="inlineStr">
         <is>
@@ -2182,7 +2188,7 @@
       </c>
       <c r="DI81" s="5" t="n"/>
     </row>
-    <row r="82" ht="4.96" customHeight="1">
+    <row r="82" ht="4.65" customHeight="1">
       <c r="L82" s="5" t="n"/>
       <c r="P82" s="5" t="n"/>
       <c r="BK82" s="5" t="n"/>
@@ -2191,7 +2197,7 @@
       <c r="CT82" s="5" t="n"/>
       <c r="DI82" s="5" t="n"/>
     </row>
-    <row r="83" ht="4.96" customHeight="1">
+    <row r="83" ht="4.65" customHeight="1">
       <c r="L83" s="1" t="n"/>
       <c r="M83" s="2" t="n"/>
       <c r="N83" s="2" t="n"/>
@@ -2295,7 +2301,7 @@
       <c r="DH83" s="2" t="n"/>
       <c r="DI83" s="1" t="n"/>
     </row>
-    <row r="84" ht="4.96" customHeight="1">
+    <row r="84" ht="4.65" customHeight="1">
       <c r="L84" s="5" t="n"/>
       <c r="M84" s="22" t="inlineStr">
         <is>
@@ -2334,7 +2340,7 @@
       </c>
       <c r="DI84" s="5" t="n"/>
     </row>
-    <row r="85" ht="4.96" customHeight="1">
+    <row r="85" ht="4.65" customHeight="1">
       <c r="L85" s="5" t="n"/>
       <c r="P85" s="5" t="n"/>
       <c r="BK85" s="5" t="n"/>
@@ -2343,7 +2349,7 @@
       <c r="CT85" s="5" t="n"/>
       <c r="DI85" s="5" t="n"/>
     </row>
-    <row r="86" ht="4.96" customHeight="1">
+    <row r="86" ht="4.65" customHeight="1">
       <c r="L86" s="5" t="n"/>
       <c r="P86" s="5" t="n"/>
       <c r="BK86" s="5" t="n"/>
@@ -2352,7 +2358,7 @@
       <c r="CT86" s="5" t="n"/>
       <c r="DI86" s="5" t="n"/>
     </row>
-    <row r="87" ht="4.96" customHeight="1">
+    <row r="87" ht="4.65" customHeight="1">
       <c r="L87" s="1" t="n"/>
       <c r="M87" s="24" t="inlineStr">
         <is>
@@ -2480,7 +2486,7 @@
       <c r="DH87" s="2" t="n"/>
       <c r="DI87" s="1" t="n"/>
     </row>
-    <row r="88" ht="4.96" customHeight="1">
+    <row r="88" ht="4.65" customHeight="1">
       <c r="L88" s="5" t="n"/>
       <c r="P88" s="5" t="n"/>
       <c r="BK88" s="5" t="n"/>
@@ -2489,7 +2495,7 @@
       <c r="CT88" s="5" t="n"/>
       <c r="DI88" s="5" t="n"/>
     </row>
-    <row r="89" ht="4.96" customHeight="1">
+    <row r="89" ht="4.65" customHeight="1">
       <c r="L89" s="5" t="n"/>
       <c r="P89" s="5" t="n"/>
       <c r="BK89" s="5" t="n"/>
@@ -2498,7 +2504,7 @@
       <c r="CT89" s="5" t="n"/>
       <c r="DI89" s="5" t="n"/>
     </row>
-    <row r="90" ht="4.96" customHeight="1">
+    <row r="90" ht="4.65" customHeight="1">
       <c r="L90" s="1" t="n"/>
       <c r="M90" s="2" t="n"/>
       <c r="N90" s="2" t="n"/>
@@ -2602,7 +2608,7 @@
       <c r="DH90" s="2" t="n"/>
       <c r="DI90" s="1" t="n"/>
     </row>
-    <row r="91" ht="4.96" customHeight="1">
+    <row r="91" ht="4.65" customHeight="1">
       <c r="L91" s="5" t="n"/>
       <c r="M91" s="22" t="inlineStr">
         <is>
@@ -2616,7 +2622,7 @@
       <c r="CT91" s="5" t="n"/>
       <c r="DI91" s="5" t="n"/>
     </row>
-    <row r="92" ht="4.96" customHeight="1">
+    <row r="92" ht="4.65" customHeight="1">
       <c r="L92" s="5" t="n"/>
       <c r="P92" s="5" t="n"/>
       <c r="BK92" s="5" t="n"/>
@@ -2625,7 +2631,7 @@
       <c r="CT92" s="5" t="n"/>
       <c r="DI92" s="5" t="n"/>
     </row>
-    <row r="93" ht="4.96" customHeight="1">
+    <row r="93" ht="4.65" customHeight="1">
       <c r="L93" s="1" t="n"/>
       <c r="M93" s="2" t="n"/>
       <c r="N93" s="2" t="n"/>
@@ -2729,7 +2735,7 @@
       <c r="DH93" s="2" t="n"/>
       <c r="DI93" s="1" t="n"/>
     </row>
-    <row r="94" ht="4.96" customHeight="1">
+    <row r="94" ht="4.65" customHeight="1">
       <c r="L94" s="5" t="n"/>
       <c r="M94" s="22" t="inlineStr">
         <is>
@@ -2743,7 +2749,7 @@
       <c r="CT94" s="5" t="n"/>
       <c r="DI94" s="5" t="n"/>
     </row>
-    <row r="95" ht="4.96" customHeight="1">
+    <row r="95" ht="4.65" customHeight="1">
       <c r="L95" s="5" t="n"/>
       <c r="P95" s="5" t="n"/>
       <c r="BK95" s="5" t="n"/>
@@ -2752,7 +2758,7 @@
       <c r="CT95" s="5" t="n"/>
       <c r="DI95" s="5" t="n"/>
     </row>
-    <row r="96" ht="4.96" customHeight="1">
+    <row r="96" ht="4.65" customHeight="1">
       <c r="L96" s="5" t="n"/>
       <c r="P96" s="5" t="n"/>
       <c r="BK96" s="5" t="n"/>
@@ -2761,7 +2767,7 @@
       <c r="CT96" s="5" t="n"/>
       <c r="DI96" s="5" t="n"/>
     </row>
-    <row r="97" ht="4.96" customHeight="1">
+    <row r="97" ht="4.65" customHeight="1">
       <c r="L97" s="1" t="n"/>
       <c r="M97" s="2" t="n"/>
       <c r="N97" s="2" t="n"/>
@@ -2865,7 +2871,7 @@
       <c r="DH97" s="2" t="n"/>
       <c r="DI97" s="1" t="n"/>
     </row>
-    <row r="98" ht="4.96" customHeight="1">
+    <row r="98" ht="4.65" customHeight="1">
       <c r="L98" s="5" t="n"/>
       <c r="M98" s="22" t="inlineStr">
         <is>
@@ -2879,7 +2885,7 @@
       <c r="CT98" s="5" t="n"/>
       <c r="DI98" s="5" t="n"/>
     </row>
-    <row r="99" ht="4.96" customHeight="1">
+    <row r="99" ht="4.65" customHeight="1">
       <c r="L99" s="5" t="n"/>
       <c r="P99" s="5" t="n"/>
       <c r="BK99" s="5" t="n"/>
@@ -2888,7 +2894,7 @@
       <c r="CT99" s="5" t="n"/>
       <c r="DI99" s="5" t="n"/>
     </row>
-    <row r="100" ht="4.96" customHeight="1">
+    <row r="100" ht="4.65" customHeight="1">
       <c r="L100" s="1" t="n"/>
       <c r="M100" s="2" t="n"/>
       <c r="N100" s="2" t="n"/>
@@ -2992,7 +2998,7 @@
       <c r="DH100" s="2" t="n"/>
       <c r="DI100" s="1" t="n"/>
     </row>
-    <row r="101" ht="4.96" customHeight="1">
+    <row r="101" ht="4.65" customHeight="1">
       <c r="L101" s="5" t="n"/>
       <c r="M101" s="22" t="inlineStr">
         <is>
@@ -3006,7 +3012,7 @@
       <c r="CT101" s="5" t="n"/>
       <c r="DI101" s="5" t="n"/>
     </row>
-    <row r="102" ht="4.96" customHeight="1">
+    <row r="102" ht="4.65" customHeight="1">
       <c r="L102" s="5" t="n"/>
       <c r="P102" s="5" t="n"/>
       <c r="BK102" s="5" t="n"/>
@@ -3015,7 +3021,7 @@
       <c r="CT102" s="5" t="n"/>
       <c r="DI102" s="5" t="n"/>
     </row>
-    <row r="103" ht="4.96" customHeight="1">
+    <row r="103" ht="4.65" customHeight="1">
       <c r="L103" s="5" t="n"/>
       <c r="P103" s="5" t="n"/>
       <c r="BK103" s="5" t="n"/>
@@ -3024,7 +3030,7 @@
       <c r="CT103" s="5" t="n"/>
       <c r="DI103" s="5" t="n"/>
     </row>
-    <row r="104" ht="4.96" customHeight="1">
+    <row r="104" ht="4.65" customHeight="1">
       <c r="L104" s="1" t="n"/>
       <c r="M104" s="24" t="inlineStr">
         <is>
@@ -3132,7 +3138,7 @@
       <c r="DH104" s="2" t="n"/>
       <c r="DI104" s="1" t="n"/>
     </row>
-    <row r="105" ht="4.96" customHeight="1">
+    <row r="105" ht="4.65" customHeight="1">
       <c r="L105" s="5" t="n"/>
       <c r="P105" s="5" t="n"/>
       <c r="BK105" s="5" t="n"/>
@@ -3141,7 +3147,7 @@
       <c r="CT105" s="5" t="n"/>
       <c r="DI105" s="5" t="n"/>
     </row>
-    <row r="106" ht="4.96" customHeight="1">
+    <row r="106" ht="4.65" customHeight="1">
       <c r="L106" s="5" t="n"/>
       <c r="P106" s="5" t="n"/>
       <c r="BK106" s="5" t="n"/>
@@ -3150,7 +3156,7 @@
       <c r="CT106" s="5" t="n"/>
       <c r="DI106" s="5" t="n"/>
     </row>
-    <row r="107" ht="4.96" customHeight="1">
+    <row r="107" ht="4.65" customHeight="1">
       <c r="L107" s="1" t="n"/>
       <c r="M107" s="2" t="n"/>
       <c r="N107" s="2" t="n"/>
@@ -3254,7 +3260,7 @@
       <c r="DH107" s="2" t="n"/>
       <c r="DI107" s="1" t="n"/>
     </row>
-    <row r="108" ht="4.96" customHeight="1">
+    <row r="108" ht="4.65" customHeight="1">
       <c r="L108" s="5" t="n"/>
       <c r="M108" s="22" t="inlineStr">
         <is>
@@ -3268,7 +3274,7 @@
       <c r="CT108" s="5" t="n"/>
       <c r="DI108" s="5" t="n"/>
     </row>
-    <row r="109" ht="4.96" customHeight="1">
+    <row r="109" ht="4.65" customHeight="1">
       <c r="L109" s="5" t="n"/>
       <c r="P109" s="5" t="n"/>
       <c r="BK109" s="5" t="n"/>
@@ -3277,7 +3283,7 @@
       <c r="CT109" s="5" t="n"/>
       <c r="DI109" s="5" t="n"/>
     </row>
-    <row r="110" ht="4.96" customHeight="1">
+    <row r="110" ht="4.65" customHeight="1">
       <c r="L110" s="1" t="n"/>
       <c r="M110" s="2" t="n"/>
       <c r="N110" s="2" t="n"/>
@@ -3381,7 +3387,7 @@
       <c r="DH110" s="2" t="n"/>
       <c r="DI110" s="1" t="n"/>
     </row>
-    <row r="111" ht="4.96" customHeight="1">
+    <row r="111" ht="4.65" customHeight="1">
       <c r="L111" s="5" t="n"/>
       <c r="M111" s="22" t="inlineStr">
         <is>
@@ -3395,7 +3401,7 @@
       <c r="CT111" s="5" t="n"/>
       <c r="DI111" s="5" t="n"/>
     </row>
-    <row r="112" ht="4.96" customHeight="1">
+    <row r="112" ht="4.65" customHeight="1">
       <c r="L112" s="5" t="n"/>
       <c r="P112" s="5" t="n"/>
       <c r="BK112" s="5" t="n"/>
@@ -3404,7 +3410,7 @@
       <c r="CT112" s="5" t="n"/>
       <c r="DI112" s="5" t="n"/>
     </row>
-    <row r="113" ht="4.96" customHeight="1">
+    <row r="113" ht="4.65" customHeight="1">
       <c r="L113" s="5" t="n"/>
       <c r="P113" s="5" t="n"/>
       <c r="BK113" s="5" t="n"/>
@@ -3413,7 +3419,7 @@
       <c r="CT113" s="5" t="n"/>
       <c r="DI113" s="5" t="n"/>
     </row>
-    <row r="114" ht="4.96" customHeight="1">
+    <row r="114" ht="4.65" customHeight="1">
       <c r="K114" s="2" t="n"/>
       <c r="L114" s="1" t="n"/>
       <c r="M114" s="2" t="n"/>
@@ -3518,7 +3524,7 @@
       <c r="DH114" s="2" t="n"/>
       <c r="DI114" s="1" t="n"/>
     </row>
-    <row r="115" ht="4.96" customHeight="1">
+    <row r="115" ht="4.65" customHeight="1">
       <c r="L115" s="5" t="n"/>
       <c r="M115" s="22" t="inlineStr">
         <is>
@@ -3532,7 +3538,7 @@
       <c r="CT115" s="5" t="n"/>
       <c r="DI115" s="5" t="n"/>
     </row>
-    <row r="116" ht="4.96" customHeight="1">
+    <row r="116" ht="4.65" customHeight="1">
       <c r="L116" s="5" t="n"/>
       <c r="P116" s="5" t="n"/>
       <c r="BK116" s="5" t="n"/>
@@ -3541,7 +3547,7 @@
       <c r="CT116" s="5" t="n"/>
       <c r="DI116" s="5" t="n"/>
     </row>
-    <row r="117" ht="4.96" customHeight="1">
+    <row r="117" ht="4.65" customHeight="1">
       <c r="L117" s="1" t="n"/>
       <c r="M117" s="2" t="n"/>
       <c r="N117" s="2" t="n"/>
@@ -3645,7 +3651,7 @@
       <c r="DH117" s="2" t="n"/>
       <c r="DI117" s="1" t="n"/>
     </row>
-    <row r="118" ht="4.96" customHeight="1">
+    <row r="118" ht="4.65" customHeight="1">
       <c r="L118" s="5" t="n"/>
       <c r="M118" s="22" t="inlineStr">
         <is>
@@ -3659,7 +3665,7 @@
       <c r="CT118" s="5" t="n"/>
       <c r="DI118" s="5" t="n"/>
     </row>
-    <row r="119" ht="4.96" customHeight="1">
+    <row r="119" ht="4.65" customHeight="1">
       <c r="L119" s="5" t="n"/>
       <c r="P119" s="5" t="n"/>
       <c r="BK119" s="5" t="n"/>
@@ -3668,7 +3674,7 @@
       <c r="CT119" s="5" t="n"/>
       <c r="DI119" s="5" t="n"/>
     </row>
-    <row r="120" ht="4.96" customHeight="1">
+    <row r="120" ht="4.65" customHeight="1">
       <c r="L120" s="5" t="n"/>
       <c r="P120" s="5" t="n"/>
       <c r="BK120" s="5" t="n"/>
@@ -3677,7 +3683,7 @@
       <c r="CT120" s="5" t="n"/>
       <c r="DI120" s="5" t="n"/>
     </row>
-    <row r="121" ht="4.96" customHeight="1">
+    <row r="121" ht="4.65" customHeight="1">
       <c r="K121" s="2" t="n"/>
       <c r="L121" s="1" t="n"/>
       <c r="M121" s="2" t="n"/>
@@ -3782,7 +3788,7 @@
       <c r="DH121" s="2" t="n"/>
       <c r="DI121" s="1" t="n"/>
     </row>
-    <row r="122" ht="4.96" customHeight="1">
+    <row r="122" ht="4.65" customHeight="1">
       <c r="L122" s="5" t="n"/>
       <c r="M122" s="22" t="inlineStr">
         <is>
@@ -3796,7 +3802,7 @@
       <c r="CT122" s="5" t="n"/>
       <c r="DI122" s="5" t="n"/>
     </row>
-    <row r="123" ht="4.96" customHeight="1">
+    <row r="123" ht="4.65" customHeight="1">
       <c r="L123" s="5" t="n"/>
       <c r="P123" s="5" t="n"/>
       <c r="BK123" s="5" t="n"/>
@@ -3805,7 +3811,7 @@
       <c r="CT123" s="5" t="n"/>
       <c r="DI123" s="5" t="n"/>
     </row>
-    <row r="124" ht="4.96" customHeight="1">
+    <row r="124" ht="4.65" customHeight="1">
       <c r="K124" s="2" t="n"/>
       <c r="L124" s="1" t="n"/>
       <c r="M124" s="2" t="n"/>
@@ -3910,7 +3916,7 @@
       <c r="DH124" s="2" t="n"/>
       <c r="DI124" s="1" t="n"/>
     </row>
-    <row r="125" ht="4.96" customHeight="1">
+    <row r="125" ht="4.65" customHeight="1">
       <c r="L125" s="5" t="n"/>
       <c r="M125" s="22" t="inlineStr">
         <is>
@@ -3924,7 +3930,7 @@
       <c r="CT125" s="5" t="n"/>
       <c r="DI125" s="5" t="n"/>
     </row>
-    <row r="126" ht="4.96" customHeight="1">
+    <row r="126" ht="4.65" customHeight="1">
       <c r="L126" s="5" t="n"/>
       <c r="P126" s="5" t="n"/>
       <c r="BK126" s="5" t="n"/>
@@ -3933,7 +3939,7 @@
       <c r="CT126" s="5" t="n"/>
       <c r="DI126" s="5" t="n"/>
     </row>
-    <row r="127" ht="4.96" customHeight="1">
+    <row r="127" ht="4.65" customHeight="1">
       <c r="L127" s="5" t="n"/>
       <c r="P127" s="5" t="n"/>
       <c r="BK127" s="5" t="n"/>
@@ -3942,7 +3948,7 @@
       <c r="CT127" s="5" t="n"/>
       <c r="DI127" s="5" t="n"/>
     </row>
-    <row r="128" ht="4.96" customHeight="1">
+    <row r="128" ht="4.65" customHeight="1">
       <c r="L128" s="1" t="n"/>
       <c r="M128" s="24" t="inlineStr">
         <is>
@@ -4050,7 +4056,7 @@
       <c r="DH128" s="2" t="n"/>
       <c r="DI128" s="1" t="n"/>
     </row>
-    <row r="129" ht="4.96" customHeight="1">
+    <row r="129" ht="4.65" customHeight="1">
       <c r="L129" s="5" t="n"/>
       <c r="P129" s="5" t="n"/>
       <c r="BK129" s="5" t="n"/>
@@ -4059,7 +4065,7 @@
       <c r="CT129" s="5" t="n"/>
       <c r="DI129" s="5" t="n"/>
     </row>
-    <row r="130" ht="4.96" customHeight="1">
+    <row r="130" ht="4.65" customHeight="1">
       <c r="L130" s="5" t="n"/>
       <c r="P130" s="5" t="n"/>
       <c r="BK130" s="5" t="n"/>
@@ -4068,7 +4074,7 @@
       <c r="CT130" s="5" t="n"/>
       <c r="DI130" s="5" t="n"/>
     </row>
-    <row r="131" ht="4.96" customHeight="1">
+    <row r="131" ht="4.65" customHeight="1">
       <c r="L131" s="1" t="n"/>
       <c r="M131" s="2" t="n"/>
       <c r="N131" s="2" t="n"/>
@@ -4172,7 +4178,7 @@
       <c r="DH131" s="2" t="n"/>
       <c r="DI131" s="1" t="n"/>
     </row>
-    <row r="132" ht="4.96" customHeight="1">
+    <row r="132" ht="4.65" customHeight="1">
       <c r="L132" s="5" t="n"/>
       <c r="M132" s="22" t="inlineStr">
         <is>
@@ -4186,7 +4192,7 @@
       <c r="CT132" s="5" t="n"/>
       <c r="DI132" s="5" t="n"/>
     </row>
-    <row r="133" ht="4.96" customHeight="1">
+    <row r="133" ht="4.65" customHeight="1">
       <c r="L133" s="5" t="n"/>
       <c r="P133" s="5" t="n"/>
       <c r="BK133" s="5" t="n"/>
@@ -4195,7 +4201,7 @@
       <c r="CT133" s="5" t="n"/>
       <c r="DI133" s="5" t="n"/>
     </row>
-    <row r="134" ht="4.96" customHeight="1">
+    <row r="134" ht="4.65" customHeight="1">
       <c r="K134" s="2" t="n"/>
       <c r="L134" s="1" t="n"/>
       <c r="M134" s="2" t="n"/>
@@ -4300,7 +4306,7 @@
       <c r="DH134" s="2" t="n"/>
       <c r="DI134" s="1" t="n"/>
     </row>
-    <row r="135" ht="4.96" customHeight="1">
+    <row r="135" ht="4.65" customHeight="1">
       <c r="L135" s="5" t="n"/>
       <c r="M135" s="22" t="inlineStr">
         <is>
@@ -4314,7 +4320,7 @@
       <c r="CT135" s="5" t="n"/>
       <c r="DI135" s="5" t="n"/>
     </row>
-    <row r="136" ht="4.96" customHeight="1">
+    <row r="136" ht="4.65" customHeight="1">
       <c r="L136" s="5" t="n"/>
       <c r="P136" s="5" t="n"/>
       <c r="BK136" s="5" t="n"/>
@@ -4323,7 +4329,7 @@
       <c r="CT136" s="5" t="n"/>
       <c r="DI136" s="5" t="n"/>
     </row>
-    <row r="137" ht="4.96" customHeight="1">
+    <row r="137" ht="4.65" customHeight="1">
       <c r="L137" s="5" t="n"/>
       <c r="P137" s="5" t="n"/>
       <c r="BK137" s="5" t="n"/>
@@ -4332,7 +4338,7 @@
       <c r="CT137" s="5" t="n"/>
       <c r="DI137" s="5" t="n"/>
     </row>
-    <row r="138" ht="4.96" customHeight="1">
+    <row r="138" ht="4.65" customHeight="1">
       <c r="K138" s="2" t="n"/>
       <c r="L138" s="1" t="n"/>
       <c r="M138" s="2" t="n"/>
@@ -4437,7 +4443,7 @@
       <c r="DH138" s="2" t="n"/>
       <c r="DI138" s="1" t="n"/>
     </row>
-    <row r="139" ht="4.96" customHeight="1">
+    <row r="139" ht="4.65" customHeight="1">
       <c r="L139" s="5" t="n"/>
       <c r="M139" s="22" t="inlineStr">
         <is>
@@ -4451,7 +4457,7 @@
       <c r="CT139" s="5" t="n"/>
       <c r="DI139" s="5" t="n"/>
     </row>
-    <row r="140" ht="4.96" customHeight="1">
+    <row r="140" ht="4.65" customHeight="1">
       <c r="L140" s="5" t="n"/>
       <c r="P140" s="5" t="n"/>
       <c r="BK140" s="5" t="n"/>
@@ -4460,7 +4466,7 @@
       <c r="CT140" s="5" t="n"/>
       <c r="DI140" s="5" t="n"/>
     </row>
-    <row r="141" ht="4.96" customHeight="1">
+    <row r="141" ht="4.65" customHeight="1">
       <c r="L141" s="1" t="n"/>
       <c r="M141" s="2" t="n"/>
       <c r="N141" s="2" t="n"/>
@@ -4564,7 +4570,7 @@
       <c r="DH141" s="2" t="n"/>
       <c r="DI141" s="1" t="n"/>
     </row>
-    <row r="142" ht="4.96" customHeight="1">
+    <row r="142" ht="4.65" customHeight="1">
       <c r="L142" s="5" t="n"/>
       <c r="M142" s="22" t="inlineStr">
         <is>
@@ -4578,7 +4584,7 @@
       <c r="CT142" s="5" t="n"/>
       <c r="DI142" s="5" t="n"/>
     </row>
-    <row r="143" ht="4.96" customHeight="1">
+    <row r="143" ht="4.65" customHeight="1">
       <c r="L143" s="5" t="n"/>
       <c r="P143" s="5" t="n"/>
       <c r="BK143" s="5" t="n"/>
@@ -4587,7 +4593,7 @@
       <c r="CT143" s="5" t="n"/>
       <c r="DI143" s="5" t="n"/>
     </row>
-    <row r="144" ht="4.96" customHeight="1">
+    <row r="144" ht="4.65" customHeight="1">
       <c r="L144" s="5" t="n"/>
       <c r="P144" s="5" t="n"/>
       <c r="BK144" s="5" t="n"/>
@@ -4596,7 +4602,7 @@
       <c r="CT144" s="5" t="n"/>
       <c r="DI144" s="5" t="n"/>
     </row>
-    <row r="145" ht="4.96" customHeight="1">
+    <row r="145" ht="4.65" customHeight="1">
       <c r="L145" s="1" t="n"/>
       <c r="M145" s="24" t="inlineStr">
         <is>
@@ -4704,7 +4710,7 @@
       <c r="DH145" s="2" t="n"/>
       <c r="DI145" s="1" t="n"/>
     </row>
-    <row r="146" ht="4.96" customHeight="1">
+    <row r="146" ht="4.65" customHeight="1">
       <c r="L146" s="5" t="n"/>
       <c r="P146" s="5" t="n"/>
       <c r="BK146" s="5" t="n"/>
@@ -4713,7 +4719,7 @@
       <c r="CT146" s="5" t="n"/>
       <c r="DI146" s="5" t="n"/>
     </row>
-    <row r="147" ht="4.96" customHeight="1">
+    <row r="147" ht="4.65" customHeight="1">
       <c r="L147" s="5" t="n"/>
       <c r="P147" s="5" t="n"/>
       <c r="BK147" s="5" t="n"/>
@@ -4722,7 +4728,7 @@
       <c r="CT147" s="5" t="n"/>
       <c r="DI147" s="5" t="n"/>
     </row>
-    <row r="148" ht="4.96" customHeight="1">
+    <row r="148" ht="4.65" customHeight="1">
       <c r="L148" s="27" t="n"/>
       <c r="M148" s="19" t="n"/>
       <c r="N148" s="19" t="n"/>
@@ -4834,15 +4840,15 @@
       <c r="DH148" s="19" t="n"/>
       <c r="DI148" s="27" t="n"/>
     </row>
-    <row r="149" ht="4.96" customHeight="1">
+    <row r="149" ht="4.65" customHeight="1">
       <c r="L149" s="5" t="n"/>
       <c r="DI149" s="5" t="n"/>
     </row>
-    <row r="150" ht="4.96" customHeight="1">
+    <row r="150" ht="4.65" customHeight="1">
       <c r="L150" s="5" t="n"/>
       <c r="DI150" s="5" t="n"/>
     </row>
-    <row r="151" ht="4.96" customHeight="1">
+    <row r="151" ht="4.65" customHeight="1">
       <c r="L151" s="1" t="n"/>
       <c r="M151" s="2" t="n"/>
       <c r="N151" s="2" t="n"/>
@@ -4946,7 +4952,7 @@
       <c r="DH151" s="2" t="n"/>
       <c r="DI151" s="1" t="n"/>
     </row>
-    <row r="152" ht="4.96" customHeight="1">
+    <row r="152" ht="4.65" customHeight="1">
       <c r="L152" s="1" t="n"/>
       <c r="M152" s="30" t="inlineStr">
         <is>
@@ -5054,15 +5060,15 @@
       <c r="DH152" s="2" t="n"/>
       <c r="DI152" s="1" t="n"/>
     </row>
-    <row r="153" ht="4.96" customHeight="1">
+    <row r="153" ht="4.65" customHeight="1">
       <c r="L153" s="5" t="n"/>
       <c r="DI153" s="5" t="n"/>
     </row>
-    <row r="154" ht="4.96" customHeight="1">
+    <row r="154" ht="4.65" customHeight="1">
       <c r="L154" s="5" t="n"/>
       <c r="DI154" s="5" t="n"/>
     </row>
-    <row r="155" ht="4.96" customHeight="1">
+    <row r="155" ht="4.65" customHeight="1">
       <c r="L155" s="31" t="inlineStr">
         <is>
           <t>・消費税は別途計上させていただきます。</t>
@@ -5170,15 +5176,15 @@
       <c r="DH155" s="2" t="n"/>
       <c r="DI155" s="1" t="n"/>
     </row>
-    <row r="156" ht="4.96" customHeight="1">
+    <row r="156" ht="4.65" customHeight="1">
       <c r="L156" s="5" t="n"/>
       <c r="DI156" s="5" t="n"/>
     </row>
-    <row r="157" ht="4.96" customHeight="1">
+    <row r="157" ht="4.65" customHeight="1">
       <c r="L157" s="5" t="n"/>
       <c r="DI157" s="5" t="n"/>
     </row>
-    <row r="158" ht="4.96" customHeight="1">
+    <row r="158" ht="4.65" customHeight="1">
       <c r="L158" s="32" t="inlineStr">
         <is>
           <t>・製品の瑕疵、無償保証期間は御購入後3ヶ月間です。</t>
@@ -5186,31 +5192,31 @@
       </c>
       <c r="DI158" s="5" t="n"/>
     </row>
-    <row r="159" ht="4.96" customHeight="1">
+    <row r="159" ht="4.65" customHeight="1">
       <c r="L159" s="5" t="n"/>
       <c r="DI159" s="5" t="n"/>
     </row>
-    <row r="160" ht="4.96" customHeight="1">
+    <row r="160" ht="4.65" customHeight="1">
       <c r="L160" s="5" t="n"/>
       <c r="DI160" s="5" t="n"/>
     </row>
-    <row r="161" ht="4.96" customHeight="1">
+    <row r="161" ht="4.65" customHeight="1">
       <c r="L161" s="5" t="n"/>
       <c r="DI161" s="5" t="n"/>
     </row>
-    <row r="162" ht="4.96" customHeight="1">
+    <row r="162" ht="4.65" customHeight="1">
       <c r="L162" s="5" t="n"/>
       <c r="DI162" s="5" t="n"/>
     </row>
-    <row r="163" ht="4.96" customHeight="1">
+    <row r="163" ht="4.65" customHeight="1">
       <c r="L163" s="5" t="n"/>
       <c r="DI163" s="5" t="n"/>
     </row>
-    <row r="164" ht="4.96" customHeight="1">
+    <row r="164" ht="4.65" customHeight="1">
       <c r="L164" s="5" t="n"/>
       <c r="DI164" s="5" t="n"/>
     </row>
-    <row r="165" ht="4.96" customHeight="1">
+    <row r="165" ht="4.65" customHeight="1">
       <c r="L165" s="1" t="n"/>
       <c r="M165" s="2" t="n"/>
       <c r="N165" s="2" t="n"/>
@@ -5314,19 +5320,25 @@
       <c r="DH165" s="2" t="n"/>
       <c r="DI165" s="1" t="n"/>
     </row>
-    <row r="166" ht="4.96" customHeight="1"/>
-    <row r="167" ht="4.96" customHeight="1"/>
-    <row r="168" ht="4.96" customHeight="1"/>
-    <row r="169" ht="4.96" customHeight="1"/>
-    <row r="170" ht="4.96" customHeight="1"/>
-    <row r="171" ht="4.96" customHeight="1"/>
-    <row r="172" ht="4.96" customHeight="1"/>
-    <row r="173" ht="4.96" customHeight="1"/>
-    <row r="174" ht="4.96" customHeight="1"/>
-    <row r="175" ht="4.96" customHeight="1"/>
-    <row r="176" ht="4.96" customHeight="1"/>
+    <row r="166" ht="4.65" customHeight="1"/>
+    <row r="167" ht="4.65" customHeight="1"/>
+    <row r="168" ht="4.65" customHeight="1"/>
+    <row r="169" ht="4.65" customHeight="1"/>
+    <row r="170" ht="4.65" customHeight="1"/>
+    <row r="171" ht="4.65" customHeight="1"/>
+    <row r="172" ht="4.65" customHeight="1"/>
+    <row r="173" ht="4.65" customHeight="1"/>
+    <row r="174" ht="4.65" customHeight="1"/>
+    <row r="175" ht="4.65" customHeight="1"/>
+    <row r="176" ht="4.65" customHeight="1"/>
+    <row r="177" ht="4.65" customHeight="1"/>
+    <row r="178" ht="4.65" customHeight="1"/>
+    <row r="179" ht="4.65" customHeight="1"/>
+    <row r="180" ht="4.65" customHeight="1"/>
+    <row r="181" ht="4.65" customHeight="1"/>
+    <row r="182" ht="4.65" customHeight="1"/>
   </sheetData>
-  <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.2" right="0.2" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
@@ -5518,7 +5530,7 @@
       </c>
       <c r="B15" s="35" t="inlineStr">
         <is>
-          <t>AAAAAA+MS-PGothic</t>
+          <t>MS-PGothic</t>
         </is>
       </c>
       <c r="C15" s="35" t="n">
@@ -5531,7 +5543,7 @@
       </c>
       <c r="B16" s="35" t="inlineStr">
         <is>
-          <t>AAAAAA+MS-PGothic</t>
+          <t>MS-PGothic</t>
         </is>
       </c>
       <c r="C16" s="35" t="n">

</xml_diff>